<commit_message>
deploy: auto-publish via publish-to-github.bat
</commit_message>
<xml_diff>
--- a/法宝属性.xlsx
+++ b/法宝属性.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="20010" windowHeight="16755"/>
+    <workbookView windowWidth="20010" windowHeight="16755" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="金" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1893" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1899" uniqueCount="197">
   <si>
     <t>法宝名</t>
   </si>
@@ -601,6 +601,9 @@
   </si>
   <si>
     <t>真武神镯</t>
+  </si>
+  <si>
+    <t>无相无我</t>
   </si>
   <si>
     <t>邪源珠</t>
@@ -1281,8 +1284,9 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
@@ -2654,7 +2658,7 @@
       <c r="G32">
         <v>0</v>
       </c>
-      <c r="H32" s="1" t="s">
+      <c r="H32" s="2" t="s">
         <v>16</v>
       </c>
       <c r="I32" t="s">
@@ -2689,13 +2693,13 @@
       <c r="G33">
         <v>0</v>
       </c>
-      <c r="H33" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="I33" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="J33" s="1" t="s">
+      <c r="H33" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="J33" s="2" t="s">
         <v>30</v>
       </c>
       <c r="K33" t="s">
@@ -3108,13 +3112,13 @@
       <c r="G46">
         <v>15</v>
       </c>
-      <c r="H46" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I46" s="1" t="s">
+      <c r="H46" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I46" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="J46" s="1" t="s">
+      <c r="J46" s="2" t="s">
         <v>30</v>
       </c>
       <c r="K46" t="s">
@@ -3143,13 +3147,13 @@
       <c r="G47">
         <v>15</v>
       </c>
-      <c r="H47" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I47" s="1" t="s">
+      <c r="H47" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I47" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="J47" s="1" t="s">
+      <c r="J47" s="2" t="s">
         <v>30</v>
       </c>
       <c r="K47" t="s">
@@ -3157,9 +3161,9 @@
       </c>
     </row>
     <row r="48" spans="1:11">
-      <c r="H48" s="1"/>
-      <c r="I48" s="1"/>
-      <c r="J48" s="1"/>
+      <c r="H48" s="2"/>
+      <c r="I48" s="2"/>
+      <c r="J48" s="2"/>
     </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:K47" etc:filterBottomFollowUsedRange="0">
@@ -3168,7 +3172,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A34:K44 A45 C45:K45 I32:K32 A32:G32 A1:K31 A46:G46 K46" numberStoredAsText="1"/>
+    <ignoredError sqref="K46 A46:G46 A1:K31 A32:G32 I32:K32 C45:K45 A45 A34:K44" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -10541,7 +10545,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K45"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1" spans="1:11">
@@ -11944,7 +11948,7 @@
       <c r="G45">
         <v>60</v>
       </c>
-      <c r="H45" t="s">
+      <c r="H45" s="1" t="s">
         <v>29</v>
       </c>
       <c r="I45" t="s">
@@ -11954,6 +11958,41 @@
         <v>30</v>
       </c>
       <c r="K45" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11">
+      <c r="A46" t="s">
+        <v>176</v>
+      </c>
+      <c r="B46" t="s">
+        <v>51</v>
+      </c>
+      <c r="C46">
+        <v>64</v>
+      </c>
+      <c r="D46">
+        <v>118</v>
+      </c>
+      <c r="E46">
+        <v>19</v>
+      </c>
+      <c r="F46">
+        <v>6400</v>
+      </c>
+      <c r="G46">
+        <v>60</v>
+      </c>
+      <c r="H46" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I46" t="s">
+        <v>5</v>
+      </c>
+      <c r="J46" t="s">
+        <v>30</v>
+      </c>
+      <c r="K46" t="s">
         <v>86</v>
       </c>
     </row>
@@ -11964,7 +12003,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A1:K45" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:K44 A45:G45 I45:K45" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -12012,7 +12051,7 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B2" t="s">
         <v>12</v>
@@ -12042,15 +12081,15 @@
         <v>15</v>
       </c>
       <c r="K2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C3">
         <v>4</v>
@@ -12077,15 +12116,15 @@
         <v>17</v>
       </c>
       <c r="K3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C4">
         <v>8</v>
@@ -12112,15 +12151,15 @@
         <v>18</v>
       </c>
       <c r="K4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C5">
         <v>16</v>
@@ -12147,12 +12186,12 @@
         <v>19</v>
       </c>
       <c r="K5" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B6" t="s">
         <v>24</v>
@@ -12170,7 +12209,7 @@
         <v>175</v>
       </c>
       <c r="G6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H6" t="s">
         <v>16</v>
@@ -12187,10 +12226,10 @@
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B7" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C7">
         <v>6</v>
@@ -12205,7 +12244,7 @@
         <v>470</v>
       </c>
       <c r="G7" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H7" t="s">
         <v>16</v>
@@ -12222,10 +12261,10 @@
     </row>
     <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B8" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C8">
         <v>12</v>
@@ -12240,7 +12279,7 @@
         <v>970</v>
       </c>
       <c r="G8" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H8" t="s">
         <v>16</v>
@@ -12257,10 +12296,10 @@
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B9" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C9">
         <v>24</v>
@@ -12275,7 +12314,7 @@
         <v>1920</v>
       </c>
       <c r="G9" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H9" t="s">
         <v>16</v>
@@ -12292,7 +12331,7 @@
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B10" t="s">
         <v>32</v>
@@ -12310,7 +12349,7 @@
         <v>138</v>
       </c>
       <c r="G10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H10" t="s">
         <v>16</v>
@@ -12327,10 +12366,10 @@
     </row>
     <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B11" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C11">
         <v>8</v>
@@ -12345,7 +12384,7 @@
         <v>455</v>
       </c>
       <c r="G11" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H11" t="s">
         <v>16</v>
@@ -12362,10 +12401,10 @@
     </row>
     <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B12" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C12">
         <v>16</v>
@@ -12380,7 +12419,7 @@
         <v>1105</v>
       </c>
       <c r="G12" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H12" t="s">
         <v>16</v>
@@ -12397,10 +12436,10 @@
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C13">
         <v>32</v>
@@ -12415,7 +12454,7 @@
         <v>2255</v>
       </c>
       <c r="G13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H13" t="s">
         <v>16</v>
@@ -12432,7 +12471,7 @@
     </row>
     <row r="14" spans="1:11">
       <c r="A14" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B14" t="s">
         <v>38</v>
@@ -12467,10 +12506,10 @@
     </row>
     <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B15" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C15">
         <v>10</v>
@@ -12502,10 +12541,10 @@
     </row>
     <row r="16" spans="1:11">
       <c r="A16" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B16" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C16">
         <v>20</v>
@@ -12537,10 +12576,10 @@
     </row>
     <row r="17" spans="1:11">
       <c r="A17" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B17" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C17">
         <v>40</v>
@@ -12572,7 +12611,7 @@
     </row>
     <row r="18" spans="1:11">
       <c r="A18" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B18" t="s">
         <v>27</v>
@@ -12590,7 +12629,7 @@
         <v>38</v>
       </c>
       <c r="G18" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H18" t="s">
         <v>16</v>
@@ -12602,15 +12641,15 @@
         <v>15</v>
       </c>
       <c r="K18" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="19" spans="1:11">
       <c r="A19" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B19" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C19">
         <v>8</v>
@@ -12625,7 +12664,7 @@
         <v>305</v>
       </c>
       <c r="G19" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H19" t="s">
         <v>16</v>
@@ -12637,15 +12676,15 @@
         <v>17</v>
       </c>
       <c r="K19" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B20" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C20">
         <v>16</v>
@@ -12660,7 +12699,7 @@
         <v>855</v>
       </c>
       <c r="G20" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H20" t="s">
         <v>16</v>
@@ -12672,15 +12711,15 @@
         <v>18</v>
       </c>
       <c r="K20" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B21" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C21">
         <v>32</v>
@@ -12695,7 +12734,7 @@
         <v>1905</v>
       </c>
       <c r="G21" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H21" t="s">
         <v>16</v>
@@ -12707,12 +12746,12 @@
         <v>19</v>
       </c>
       <c r="K21" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B22" t="s">
         <v>46</v>
@@ -12742,15 +12781,15 @@
         <v>15</v>
       </c>
       <c r="K22" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B23" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C23">
         <v>10</v>
@@ -12777,15 +12816,15 @@
         <v>17</v>
       </c>
       <c r="K23" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B24" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C24">
         <v>20</v>
@@ -12812,15 +12851,15 @@
         <v>18</v>
       </c>
       <c r="K24" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B25" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C25">
         <v>40</v>
@@ -12847,12 +12886,12 @@
         <v>19</v>
       </c>
       <c r="K25" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="26" spans="1:11">
       <c r="A26" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B26" t="s">
         <v>36</v>
@@ -12870,7 +12909,7 @@
         <v>238</v>
       </c>
       <c r="G26" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H26" t="s">
         <v>16</v>
@@ -12887,10 +12926,10 @@
     </row>
     <row r="27" spans="1:11">
       <c r="A27" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B27" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C27">
         <v>8</v>
@@ -12905,7 +12944,7 @@
         <v>555</v>
       </c>
       <c r="G27" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H27" t="s">
         <v>16</v>
@@ -12922,10 +12961,10 @@
     </row>
     <row r="28" spans="1:11">
       <c r="A28" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B28" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C28">
         <v>16</v>
@@ -12940,7 +12979,7 @@
         <v>1255</v>
       </c>
       <c r="G28" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H28" t="s">
         <v>16</v>
@@ -12957,10 +12996,10 @@
     </row>
     <row r="29" spans="1:11">
       <c r="A29" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B29" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C29">
         <v>32</v>
@@ -12975,7 +13014,7 @@
         <v>2505</v>
       </c>
       <c r="G29" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H29" t="s">
         <v>16</v>
@@ -12992,7 +13031,7 @@
     </row>
     <row r="30" spans="1:11">
       <c r="A30" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B30" t="s">
         <v>43</v>
@@ -13027,10 +13066,10 @@
     </row>
     <row r="31" spans="1:11">
       <c r="A31" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B31" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C31">
         <v>10</v>
@@ -13062,10 +13101,10 @@
     </row>
     <row r="32" spans="1:11">
       <c r="A32" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B32" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C32">
         <v>20</v>
@@ -13097,10 +13136,10 @@
     </row>
     <row r="33" spans="1:11">
       <c r="A33" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B33" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C33">
         <v>40</v>
@@ -13132,7 +13171,7 @@
     </row>
     <row r="34" spans="1:11">
       <c r="A34" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B34" t="s">
         <v>21</v>
@@ -13150,7 +13189,7 @@
         <v>125</v>
       </c>
       <c r="G34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H34" t="s">
         <v>16</v>
@@ -13167,10 +13206,10 @@
     </row>
     <row r="35" spans="1:11">
       <c r="A35" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B35" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C35">
         <v>6</v>
@@ -13185,7 +13224,7 @@
         <v>370</v>
       </c>
       <c r="G35" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H35" t="s">
         <v>16</v>
@@ -13202,10 +13241,10 @@
     </row>
     <row r="36" spans="1:11">
       <c r="A36" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B36" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C36">
         <v>12</v>
@@ -13220,7 +13259,7 @@
         <v>820</v>
       </c>
       <c r="G36" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H36" t="s">
         <v>16</v>
@@ -13237,10 +13276,10 @@
     </row>
     <row r="37" spans="1:11">
       <c r="A37" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B37" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C37">
         <v>24</v>
@@ -13255,7 +13294,7 @@
         <v>1670</v>
       </c>
       <c r="G37" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H37" t="s">
         <v>16</v>
@@ -13272,7 +13311,7 @@
     </row>
     <row r="38" spans="1:11">
       <c r="A38" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B38" t="s">
         <v>38</v>
@@ -13290,7 +13329,7 @@
         <v>4700</v>
       </c>
       <c r="G38" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H38" t="s">
         <v>16</v>
@@ -13307,7 +13346,7 @@
     </row>
     <row r="39" spans="1:11">
       <c r="A39" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B39" t="s">
         <v>53</v>
@@ -13342,7 +13381,7 @@
     </row>
     <row r="40" spans="1:11">
       <c r="A40" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B40" t="s">
         <v>46</v>
@@ -13360,7 +13399,7 @@
         <v>4250</v>
       </c>
       <c r="G40" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H40" t="s">
         <v>16</v>
@@ -13372,12 +13411,12 @@
         <v>30</v>
       </c>
       <c r="K40" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="41" spans="1:11">
       <c r="A41" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B41" t="s">
         <v>51</v>
@@ -13407,12 +13446,12 @@
         <v>30</v>
       </c>
       <c r="K41" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="42" spans="1:11">
       <c r="A42" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B42" t="s">
         <v>43</v>
@@ -13430,7 +13469,7 @@
         <v>5100</v>
       </c>
       <c r="G42" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H42" t="s">
         <v>16</v>
@@ -13447,7 +13486,7 @@
     </row>
     <row r="43" spans="1:11">
       <c r="A43" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B43" t="s">
         <v>49</v>
@@ -13482,7 +13521,7 @@
     </row>
     <row r="44" spans="1:11">
       <c r="A44" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B44" t="s">
         <v>32</v>
@@ -13517,7 +13556,7 @@
     </row>
     <row r="45" spans="1:11">
       <c r="A45" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B45" t="s">
         <v>27</v>
@@ -13547,7 +13586,7 @@
         <v>30</v>
       </c>
       <c r="K45" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>